<commit_message>
all plastic bead data done
</commit_message>
<xml_diff>
--- a/raw_data.xlsx
+++ b/raw_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/67293e35e6a9c6ca/Desktop/pfinal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_751D8C3155516C0F62355476585DCE3A8747A12D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D3B499E-80B5-49AE-A331-2EF99CDA5840}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_4611FDBA516F8A0F62355476585DCE3A8747A1E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0922DD7-21A0-4EA0-BF6D-35AB4C9A1F8D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
   <si>
     <t>Video Name</t>
   </si>
@@ -154,19 +154,22 @@
     <t>175 gms 150 lpm-2.avi</t>
   </si>
   <si>
+    <t>250 lpm-1.avi</t>
+  </si>
+  <si>
+    <t>300 lpm-2.avi</t>
+  </si>
+  <si>
+    <t>400  lpm-1.avi</t>
+  </si>
+  <si>
+    <t>350 lpm-2.avi</t>
+  </si>
+  <si>
+    <t>450 lpm.avi</t>
+  </si>
+  <si>
     <t>200 lpm-1.avi</t>
-  </si>
-  <si>
-    <t>250 lpm-1.avi</t>
-  </si>
-  <si>
-    <t>300 lpm-2.avi</t>
-  </si>
-  <si>
-    <t>350 lpm-2.avi</t>
-  </si>
-  <si>
-    <t>400  lpm-1.avi</t>
   </si>
 </sst>
 </file>
@@ -529,7 +532,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI14"/>
+  <dimension ref="A1:AI15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.3">
@@ -1236,7 +1239,7 @@
         <v>0.2212720829301113</v>
       </c>
       <c r="U7">
-        <v>187.19618215887411</v>
+        <v>187.196182158874</v>
       </c>
       <c r="V7">
         <v>51.923039418583677</v>
@@ -1506,79 +1509,79 @@
         <v>500</v>
       </c>
       <c r="D10">
-        <v>286</v>
+        <v>227</v>
       </c>
       <c r="E10">
-        <v>192</v>
+        <v>227</v>
       </c>
       <c r="F10">
-        <v>1111</v>
+        <v>1047</v>
       </c>
       <c r="G10">
-        <v>189</v>
+        <v>228</v>
       </c>
       <c r="H10">
         <v>100</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J10">
-        <v>258</v>
+        <v>287</v>
       </c>
       <c r="K10">
-        <v>1280</v>
+        <v>1278</v>
       </c>
       <c r="L10">
         <v>472</v>
       </c>
       <c r="M10">
-        <v>57.211742953914097</v>
+        <v>57.560932807174737</v>
       </c>
       <c r="N10">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="O10">
-        <v>18.42412061227742</v>
+        <v>15.60974449008129</v>
       </c>
       <c r="P10">
-        <v>19.030177211365501</v>
+        <v>16.585353520711369</v>
       </c>
       <c r="Q10">
-        <v>129</v>
+        <v>70</v>
       </c>
       <c r="R10">
-        <v>422</v>
+        <v>248</v>
       </c>
       <c r="S10">
-        <v>0.58599999999999997</v>
+        <v>0.35599999999999998</v>
       </c>
       <c r="T10">
-        <v>0.79132920930253581</v>
+        <v>1.1259534650815219</v>
       </c>
       <c r="U10">
-        <v>463.71891665128601</v>
+        <v>400.83943356902188</v>
       </c>
       <c r="V10">
-        <v>57.211742953914097</v>
+        <v>56.463372647715907</v>
       </c>
       <c r="W10">
-        <v>28.187005519897461</v>
+        <v>39.224544195424407</v>
       </c>
       <c r="X10">
-        <v>-0.5359033292903691</v>
+        <v>-0.81629366910257095</v>
       </c>
       <c r="Y10">
-        <v>1.2966</v>
+        <v>1.6012</v>
       </c>
       <c r="Z10">
         <v>2453407.21</v>
       </c>
       <c r="AA10">
-        <v>0.3322</v>
+        <v>0.63680000000000003</v>
       </c>
       <c r="AB10">
-        <v>0.83609999999999995</v>
+        <v>1.0719000000000001</v>
       </c>
       <c r="AC10">
         <v>1.1616</v>
@@ -1590,16 +1593,16 @@
         <v>0.43530000000000002</v>
       </c>
       <c r="AF10">
-        <v>0.29089999999999999</v>
+        <v>0.23860000000000001</v>
       </c>
       <c r="AG10">
-        <v>12.01</v>
+        <v>15.53</v>
       </c>
       <c r="AH10">
-        <v>2947.54</v>
+        <v>1983.15</v>
       </c>
       <c r="AI10">
-        <v>16711.259999999998</v>
+        <v>10069.08</v>
       </c>
     </row>
     <row r="11" spans="1:35" x14ac:dyDescent="0.3">
@@ -1613,79 +1616,79 @@
         <v>500</v>
       </c>
       <c r="D11">
-        <v>227</v>
+        <v>260</v>
       </c>
       <c r="E11">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F11">
-        <v>1047</v>
+        <v>1087</v>
       </c>
       <c r="G11">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="H11">
         <v>100</v>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J11">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K11">
-        <v>1278</v>
+        <v>1280</v>
       </c>
       <c r="L11">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="M11">
-        <v>57.560932807174737</v>
+        <v>57.434460128068302</v>
       </c>
       <c r="N11">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="O11">
-        <v>15.60974449008129</v>
+        <v>13.300611819131611</v>
       </c>
       <c r="P11">
-        <v>16.585353520711369</v>
+        <v>11.849635984317249</v>
       </c>
       <c r="Q11">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="R11">
-        <v>248</v>
+        <v>230</v>
       </c>
       <c r="S11">
-        <v>0.35599999999999998</v>
+        <v>0.26800000000000002</v>
       </c>
       <c r="T11">
-        <v>1.1259534650815219</v>
+        <v>1.320111959107837</v>
       </c>
       <c r="U11">
-        <v>400.83943356902188</v>
+        <v>353.79000504090033</v>
       </c>
       <c r="V11">
-        <v>56.463372647715907</v>
+        <v>56.346228251957527</v>
       </c>
       <c r="W11">
-        <v>39.224544195424407</v>
+        <v>41.703934753801832</v>
       </c>
       <c r="X11">
-        <v>-0.81629366910257095</v>
+        <v>-0.89109069725055678</v>
       </c>
       <c r="Y11">
-        <v>1.6012</v>
+        <v>1.9298999999999999</v>
       </c>
       <c r="Z11">
         <v>2453407.21</v>
       </c>
       <c r="AA11">
-        <v>0.63680000000000003</v>
+        <v>0.96550000000000002</v>
       </c>
       <c r="AB11">
-        <v>1.0719000000000001</v>
+        <v>1.3263</v>
       </c>
       <c r="AC11">
         <v>1.1616</v>
@@ -1697,16 +1700,16 @@
         <v>0.43530000000000002</v>
       </c>
       <c r="AF11">
-        <v>0.23860000000000001</v>
+        <v>0.14879999999999999</v>
       </c>
       <c r="AG11">
-        <v>15.53</v>
+        <v>18.53</v>
       </c>
       <c r="AH11">
-        <v>1983.15</v>
+        <v>1760.49</v>
       </c>
       <c r="AI11">
-        <v>10069.08</v>
+        <v>7969.42</v>
       </c>
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.3">
@@ -1720,16 +1723,16 @@
         <v>500</v>
       </c>
       <c r="D12">
-        <v>260</v>
+        <v>373</v>
       </c>
       <c r="E12">
-        <v>228</v>
+        <v>595</v>
       </c>
       <c r="F12">
-        <v>1087</v>
+        <v>1177</v>
       </c>
       <c r="G12">
-        <v>221</v>
+        <v>595</v>
       </c>
       <c r="H12">
         <v>100</v>
@@ -1738,61 +1741,61 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>288</v>
+        <v>662</v>
       </c>
       <c r="K12">
-        <v>1280</v>
+        <v>1696</v>
       </c>
       <c r="L12">
-        <v>475</v>
+        <v>464</v>
       </c>
       <c r="M12">
-        <v>57.434460128068302</v>
+        <v>57.711442786069647</v>
       </c>
       <c r="N12">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="O12">
-        <v>13.300611819131611</v>
+        <v>10.133265</v>
       </c>
       <c r="P12">
-        <v>11.849635984317249</v>
+        <v>10.233459999999999</v>
       </c>
       <c r="Q12">
-        <v>96</v>
+        <v>13</v>
       </c>
       <c r="R12">
-        <v>230</v>
+        <v>176</v>
       </c>
       <c r="S12">
-        <v>0.26800000000000002</v>
+        <v>0.32600000000000001</v>
       </c>
       <c r="T12">
-        <v>1.320111959107837</v>
+        <v>1.5064056832992021</v>
       </c>
       <c r="U12">
-        <v>353.79000504090033</v>
+        <v>491.08825275553988</v>
       </c>
       <c r="V12">
-        <v>56.346228251957527</v>
+        <v>52.736318407960198</v>
       </c>
       <c r="W12">
-        <v>41.703934753801832</v>
+        <v>32.41545</v>
       </c>
       <c r="X12">
-        <v>-0.89109069725055678</v>
+        <v>-1.3811222938303589</v>
       </c>
       <c r="Y12">
-        <v>1.9298999999999999</v>
+        <v>2.5486</v>
       </c>
       <c r="Z12">
-        <v>2453407.21</v>
+        <v>3548972.18</v>
       </c>
       <c r="AA12">
-        <v>0.96550000000000002</v>
+        <v>1.5052000000000001</v>
       </c>
       <c r="AB12">
-        <v>1.3263</v>
+        <v>1.744</v>
       </c>
       <c r="AC12">
         <v>1.1616</v>
@@ -1804,16 +1807,16 @@
         <v>0.43530000000000002</v>
       </c>
       <c r="AF12">
-        <v>0.14879999999999999</v>
+        <v>0.1198</v>
       </c>
       <c r="AG12">
-        <v>18.53</v>
+        <v>18.36</v>
       </c>
       <c r="AH12">
-        <v>1760.49</v>
+        <v>2455.14</v>
       </c>
       <c r="AI12">
-        <v>7969.42</v>
+        <v>15216.7</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.3">
@@ -1827,79 +1830,79 @@
         <v>500</v>
       </c>
       <c r="D13">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E13">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F13">
         <v>1070</v>
       </c>
       <c r="G13">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="H13">
         <v>100</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J13">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="K13">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="L13">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="M13">
-        <v>56.657931305229681</v>
+        <v>57.402532180019882</v>
       </c>
       <c r="N13">
         <v>350</v>
       </c>
       <c r="O13">
-        <v>12.348523489601339</v>
+        <v>12.62127557446526</v>
       </c>
       <c r="P13">
-        <v>13.6802270031858</v>
+        <v>13.95621818330293</v>
       </c>
       <c r="Q13">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="R13">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="S13">
-        <v>0.26</v>
+        <v>0.246</v>
       </c>
       <c r="T13">
-        <v>1.538270527604086</v>
+        <v>1.557246900922264</v>
       </c>
       <c r="U13">
-        <v>399.95033717706218</v>
+        <v>383.08273762687702</v>
       </c>
       <c r="V13">
-        <v>55.447291747425623</v>
+        <v>51.334611230757737</v>
       </c>
       <c r="W13">
-        <v>37.366545201746561</v>
+        <v>33.361884922853442</v>
       </c>
       <c r="X13">
-        <v>-0.76363293156553202</v>
+        <v>-0.65842446439391444</v>
       </c>
       <c r="Y13">
-        <v>2.3136999999999999</v>
+        <v>2.2541000000000002</v>
       </c>
       <c r="Z13">
-        <v>2453407.21</v>
+        <v>3548972.18</v>
       </c>
       <c r="AA13">
-        <v>1.3492999999999999</v>
+        <v>1.2107000000000001</v>
       </c>
       <c r="AB13">
-        <v>1.6233</v>
+        <v>1.5161</v>
       </c>
       <c r="AC13">
         <v>1.1616</v>
@@ -1911,16 +1914,16 @@
         <v>0.43530000000000002</v>
       </c>
       <c r="AF13">
-        <v>0.18609999999999999</v>
+        <v>0.188</v>
       </c>
       <c r="AG13">
-        <v>17.61</v>
+        <v>17.78</v>
       </c>
       <c r="AH13">
-        <v>2151.58</v>
+        <v>2430.92</v>
       </c>
       <c r="AI13">
-        <v>10898.08</v>
+        <v>11333.1</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.3">
@@ -1934,16 +1937,16 @@
         <v>500</v>
       </c>
       <c r="D14">
-        <v>370</v>
+        <v>237</v>
       </c>
       <c r="E14">
-        <v>594</v>
+        <v>133</v>
       </c>
       <c r="F14">
-        <v>1178</v>
+        <v>1070</v>
       </c>
       <c r="G14">
-        <v>595</v>
+        <v>131</v>
       </c>
       <c r="H14">
         <v>100</v>
@@ -1952,61 +1955,61 @@
         <v>0</v>
       </c>
       <c r="J14">
-        <v>656</v>
+        <v>200</v>
       </c>
       <c r="K14">
-        <v>1696</v>
+        <v>1280</v>
       </c>
       <c r="L14">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="M14">
-        <v>57.796985438802487</v>
+        <v>56.30235872804559</v>
       </c>
       <c r="N14">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="O14">
-        <v>10.133265</v>
+        <v>10.924338260665561</v>
       </c>
       <c r="P14">
-        <v>10.324</v>
+        <v>14.885911476071749</v>
       </c>
       <c r="Q14">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="R14">
-        <v>176</v>
+        <v>121</v>
       </c>
       <c r="S14">
-        <v>0.32600000000000001</v>
+        <v>0.13800000000000001</v>
       </c>
       <c r="T14">
-        <v>1.4985807197098351</v>
+        <v>1.7537490056902201</v>
       </c>
       <c r="U14">
-        <v>488.53731462540628</v>
+        <v>242.01736278525041</v>
       </c>
       <c r="V14">
-        <v>51.7326336475791</v>
+        <v>51.020261107503998</v>
       </c>
       <c r="W14">
-        <v>56.255850847875642</v>
+        <v>34.134658597830651</v>
       </c>
       <c r="X14">
-        <v>-1.496936653407295</v>
+        <v>-0.67793345585744169</v>
       </c>
       <c r="Y14">
-        <v>2.5409999999999999</v>
+        <v>3.0124</v>
       </c>
       <c r="Z14">
         <v>3548972.18</v>
       </c>
       <c r="AA14">
-        <v>1.4977</v>
+        <v>1.9691000000000001</v>
       </c>
       <c r="AB14">
-        <v>1.7382</v>
+        <v>2.1031</v>
       </c>
       <c r="AC14">
         <v>1.1616</v>
@@ -2018,16 +2021,123 @@
         <v>0.43530000000000002</v>
       </c>
       <c r="AF14">
-        <v>0.11990000000000001</v>
+        <v>0.21149999999999999</v>
       </c>
       <c r="AG14">
-        <v>18.39</v>
+        <v>16.55</v>
       </c>
       <c r="AH14">
-        <v>1139.0899999999999</v>
+        <v>2614.14</v>
       </c>
       <c r="AI14">
-        <v>8389.64</v>
+        <v>7697.58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15">
+        <v>500</v>
+      </c>
+      <c r="D15">
+        <v>287</v>
+      </c>
+      <c r="E15">
+        <v>192</v>
+      </c>
+      <c r="F15">
+        <v>1114</v>
+      </c>
+      <c r="G15">
+        <v>191</v>
+      </c>
+      <c r="H15">
+        <v>100</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>255</v>
+      </c>
+      <c r="K15">
+        <v>1277</v>
+      </c>
+      <c r="L15">
+        <v>473</v>
+      </c>
+      <c r="M15">
+        <v>57.194637751420949</v>
+      </c>
+      <c r="N15">
+        <v>200</v>
+      </c>
+      <c r="O15">
+        <v>18.37967217381815</v>
+      </c>
+      <c r="P15">
+        <v>18.742428861459299</v>
+      </c>
+      <c r="Q15">
+        <v>129</v>
+      </c>
+      <c r="R15">
+        <v>421</v>
+      </c>
+      <c r="S15">
+        <v>0.58399999999999996</v>
+      </c>
+      <c r="T15">
+        <v>0.7925905339824959</v>
+      </c>
+      <c r="U15">
+        <v>462.87287184577758</v>
+      </c>
+      <c r="V15">
+        <v>51.148692957401821</v>
+      </c>
+      <c r="W15">
+        <v>27.893754066568039</v>
+      </c>
+      <c r="X15">
+        <v>-0.5293331805294158</v>
+      </c>
+      <c r="Y15">
+        <v>1.2974000000000001</v>
+      </c>
+      <c r="Z15">
+        <v>3548972.18</v>
+      </c>
+      <c r="AA15">
+        <v>0.25409999999999999</v>
+      </c>
+      <c r="AB15">
+        <v>0.77569999999999995</v>
+      </c>
+      <c r="AC15">
+        <v>1.1616</v>
+      </c>
+      <c r="AD15">
+        <v>0.13780000000000001</v>
+      </c>
+      <c r="AE15">
+        <v>0.43530000000000002</v>
+      </c>
+      <c r="AF15">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="AG15">
+        <v>12.42</v>
+      </c>
+      <c r="AH15">
+        <v>2968.82</v>
+      </c>
+      <c r="AI15">
+        <v>16783.580000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>